<commit_message>
tests(core): Regenerate golden xlsx
</commit_message>
<xml_diff>
--- a/core/tests/testcases/artificial/ortools/ex1_even_shift_distribution.prettify.xlsx
+++ b/core/tests/testcases/artificial/ortools/ex1_even_shift_distribution.prettify.xlsx
@@ -26,20 +26,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -65,24 +60,11 @@
         <color rgb="00374151"/>
       </bottom>
     </border>
-    <border>
-      <right style="medium">
-        <color rgb="009CA3AF"/>
-      </right>
-    </border>
-    <border>
-      <right style="medium">
-        <color rgb="009CA3AF"/>
-      </right>
-      <bottom style="medium">
-        <color rgb="00374151"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -90,22 +72,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -481,10 +451,10 @@
       <c r="B1" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="C1" s="3" t="n">
+      <c r="C1" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="D1" s="4" t="n">
+      <c r="D1" s="1" t="n">
         <v>20</v>
       </c>
       <c r="E1" s="2" t="inlineStr"/>
@@ -498,67 +468,67 @@
       <c r="M1" s="2" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr"/>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Fri</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Sat</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Sun</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr"/>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>OFF (Total)</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>OFF (Weekday)</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>OFF (Weekend)</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>D Count</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>E Count</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>N Count</t>
         </is>
       </c>
-      <c r="L2" s="6" t="inlineStr"/>
-      <c r="M2" s="6" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr"/>
+      <c r="M2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
         <v>0</v>
       </c>
       <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>D</t>
         </is>
@@ -594,8 +564,8 @@
           <t>E</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>E</t>
         </is>
@@ -631,12 +601,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -664,41 +634,41 @@
       <c r="M5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="6" t="inlineStr"/>
-      <c r="M6" s="6" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -709,8 +679,8 @@
       <c r="B7" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="4" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="1" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="1" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr"/>
@@ -722,33 +692,33 @@
       <c r="M7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>OPTIMAL</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr"/>
-      <c r="D8" s="8" t="inlineStr"/>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr"/>
-      <c r="J8" s="6" t="inlineStr"/>
-      <c r="K8" s="5" t="inlineStr"/>
-      <c r="L8" s="6" t="inlineStr"/>
-      <c r="M8" s="6" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="3" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="1" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="1" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr"/>
@@ -768,10 +738,10 @@
       <c r="B10" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="4" t="n">
+      <c r="C10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -793,10 +763,10 @@
       <c r="B11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="4" t="n">
+      <c r="C11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
@@ -810,29 +780,29 @@
       <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>N Count</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="6" t="inlineStr"/>
-      <c r="K12" s="5" t="inlineStr"/>
-      <c r="L12" s="6" t="inlineStr"/>
-      <c r="M12" s="6" t="inlineStr"/>
+      <c r="B12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>